<commit_message>
查战绩相关脚本的对局信息数据框结构更新【Match Information Dataframe Structure Update in Customized Programs 05 and 11】
跟进14.14版本无尽狂潮模式的更新，在对局信息数据框中添加了2个强化符文，并同步更新了自定义脚本主数据框结构工作簿。
Following the introduction of SWARM  in Patch 14.14, added 2 augments into the match information dataframes and meanwhile Customized Program Main Dataframe workbook.
</commit_message>
<xml_diff>
--- a/Customized Program Main Dataframe Structure.xlsx
+++ b/Customized Program Main Dataframe Structure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0FC01E-97E2-4DA2-8AAB-BE87616C63C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881122C6-566A-4CA0-B8DF-3D3D23E8EABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B2D932DB-2183-440F-AF66-43F3E8354BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{B2D932DB-2183-440F-AF66-43F3E8354BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="05 - mastery_header" sheetId="3" r:id="rId1"/>
@@ -28,9 +28,9 @@
     <sheet name="12 - player_loot_header" sheetId="11" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'05 - LoLGame_info_header'!$A$1:$E$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'05 - LoLGame_info_header'!$A$1:$E$146</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05 - TFTHistory_header'!$A$1:$E$160</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'11 - LoLGame_info_header'!$A$1:$E$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'11 - LoLGame_info_header'!$A$1:$E$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11 - TFTHistory_header'!$A$1:$E$160</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="1008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2377" uniqueCount="1016">
   <si>
     <t>gameCreationDate</t>
   </si>
@@ -3259,6 +3259,38 @@
   </si>
   <si>
     <t>下一级成就所需英雄成就标记个数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>playerAugment5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>playerAugment5_rarity</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>playerAugment6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>playerAugment6_rarity</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>强化符文5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>强化符文5等级</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>强化符文6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>强化符文6等级</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -5093,7 +5125,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86E653D2-5962-4B6A-AE49-EF482E17CB95}">
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E153"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
@@ -5500,7 +5532,7 @@
       </c>
       <c r="D26" s="7"/>
       <c r="E26">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5543,7 +5575,7 @@
         <v>149</v>
       </c>
       <c r="E29">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5577,7 +5609,7 @@
         <v>149</v>
       </c>
       <c r="E31">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5594,7 +5626,7 @@
         <v>149</v>
       </c>
       <c r="E32">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5611,7 +5643,7 @@
         <v>149</v>
       </c>
       <c r="E33">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5628,7 +5660,7 @@
         <v>149</v>
       </c>
       <c r="E34">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5659,7 +5691,7 @@
         <v>149</v>
       </c>
       <c r="E36">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5676,7 +5708,7 @@
         <v>149</v>
       </c>
       <c r="E37">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5693,7 +5725,7 @@
         <v>149</v>
       </c>
       <c r="E38">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5710,7 +5742,7 @@
         <v>149</v>
       </c>
       <c r="E39">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5727,7 +5759,7 @@
         <v>149</v>
       </c>
       <c r="E40">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5744,7 +5776,7 @@
         <v>149</v>
       </c>
       <c r="E41">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5761,7 +5793,7 @@
         <v>149</v>
       </c>
       <c r="E42">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5778,7 +5810,7 @@
         <v>149</v>
       </c>
       <c r="E43">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5795,7 +5827,7 @@
         <v>149</v>
       </c>
       <c r="E44">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5812,7 +5844,7 @@
         <v>149</v>
       </c>
       <c r="E45">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5829,7 +5861,7 @@
         <v>149</v>
       </c>
       <c r="E46">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5846,7 +5878,7 @@
         <v>149</v>
       </c>
       <c r="E47">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5863,7 +5895,7 @@
         <v>149</v>
       </c>
       <c r="E48">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5985,7 +6017,7 @@
         <v>149</v>
       </c>
       <c r="E56">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6016,7 +6048,7 @@
         <v>149</v>
       </c>
       <c r="E58">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6033,7 +6065,7 @@
         <v>149</v>
       </c>
       <c r="E59">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6050,7 +6082,7 @@
         <v>149</v>
       </c>
       <c r="E60">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6067,7 +6099,7 @@
         <v>149</v>
       </c>
       <c r="E61">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6084,7 +6116,7 @@
         <v>149</v>
       </c>
       <c r="E62">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6101,7 +6133,7 @@
         <v>149</v>
       </c>
       <c r="E63">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6118,7 +6150,7 @@
         <v>149</v>
       </c>
       <c r="E64">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6135,7 +6167,7 @@
         <v>149</v>
       </c>
       <c r="E65">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6152,7 +6184,7 @@
         <v>149</v>
       </c>
       <c r="E66">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6169,7 +6201,7 @@
         <v>149</v>
       </c>
       <c r="E67">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6200,7 +6232,7 @@
         <v>149</v>
       </c>
       <c r="E69">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6215,7 +6247,7 @@
       </c>
       <c r="D70" s="7"/>
       <c r="E70">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6230,7 +6262,7 @@
       </c>
       <c r="D71" s="7"/>
       <c r="E71">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6287,7 +6319,7 @@
       </c>
       <c r="D75" s="7"/>
       <c r="E75">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6302,7 +6334,7 @@
       </c>
       <c r="D76" s="7"/>
       <c r="E76">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6359,7 +6391,7 @@
       </c>
       <c r="D80" s="7"/>
       <c r="E80">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6374,7 +6406,7 @@
       </c>
       <c r="D81" s="7"/>
       <c r="E81">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6431,7 +6463,7 @@
       </c>
       <c r="D85" s="7"/>
       <c r="E85">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6446,7 +6478,7 @@
       </c>
       <c r="D86" s="7"/>
       <c r="E86">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6503,7 +6535,7 @@
       </c>
       <c r="D90" s="7"/>
       <c r="E90">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6518,7 +6550,7 @@
       </c>
       <c r="D91" s="7"/>
       <c r="E91">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6575,7 +6607,7 @@
       </c>
       <c r="D95" s="7"/>
       <c r="E95">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6590,7 +6622,7 @@
       </c>
       <c r="D96" s="7"/>
       <c r="E96">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6647,7 +6679,7 @@
       </c>
       <c r="D100" s="7"/>
       <c r="E100">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6662,7 +6694,7 @@
       </c>
       <c r="D101" s="7"/>
       <c r="E101">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6679,7 +6711,7 @@
         <v>149</v>
       </c>
       <c r="E102">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6696,7 +6728,7 @@
         <v>149</v>
       </c>
       <c r="E103">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6713,7 +6745,7 @@
         <v>149</v>
       </c>
       <c r="E104">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6841,27 +6873,29 @@
         <v>111</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>734</v>
+        <v>1008</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>744</v>
-      </c>
-      <c r="D113" s="7" t="s">
-        <v>149</v>
+        <v>1012</v>
+      </c>
+      <c r="D113" s="7"/>
+      <c r="E113">
+        <v>35</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A114" s="3">
         <v>112</v>
       </c>
-      <c r="B114" s="4" t="s">
-        <v>735</v>
+      <c r="B114" s="17" t="s">
+        <v>1009</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>745</v>
-      </c>
-      <c r="D114" s="7" t="s">
-        <v>149</v>
+        <v>1013</v>
+      </c>
+      <c r="D114" s="7"/>
+      <c r="E114">
+        <v>36</v>
       </c>
     </row>
     <row r="115" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6869,27 +6903,29 @@
         <v>113</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>736</v>
+        <v>1010</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>746</v>
-      </c>
-      <c r="D115" s="7" t="s">
-        <v>149</v>
+        <v>1014</v>
+      </c>
+      <c r="D115" s="7"/>
+      <c r="E115">
+        <v>37</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>114</v>
       </c>
-      <c r="B116" s="4" t="s">
-        <v>737</v>
+      <c r="B116" s="17" t="s">
+        <v>1011</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>747</v>
-      </c>
-      <c r="D116" s="7" t="s">
-        <v>149</v>
+        <v>1015</v>
+      </c>
+      <c r="D116" s="7"/>
+      <c r="E116">
+        <v>38</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -6897,10 +6933,10 @@
         <v>115</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="D117" s="7" t="s">
         <v>149</v>
@@ -6911,10 +6947,10 @@
         <v>116</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="D118" s="7" t="s">
         <v>149</v>
@@ -6925,10 +6961,10 @@
         <v>117</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="D119" s="7" t="s">
         <v>149</v>
@@ -6939,10 +6975,10 @@
         <v>118</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="D120" s="7" t="s">
         <v>149</v>
@@ -6953,10 +6989,10 @@
         <v>119</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="D121" s="7" t="s">
         <v>149</v>
@@ -6967,10 +7003,10 @@
         <v>120</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="D122" s="7" t="s">
         <v>149</v>
@@ -6981,28 +7017,27 @@
         <v>121</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>288</v>
+        <v>740</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D123" s="7"/>
+        <v>750</v>
+      </c>
+      <c r="D123" s="7" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="124" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A124" s="3">
         <v>122</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>50</v>
+        <v>741</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>123</v>
+        <v>751</v>
       </c>
       <c r="D124" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="E124">
-        <v>50</v>
       </c>
     </row>
     <row r="125" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7010,16 +7045,13 @@
         <v>123</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>316</v>
+        <v>742</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>124</v>
+        <v>752</v>
       </c>
       <c r="D125" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="E125">
-        <v>76</v>
       </c>
     </row>
     <row r="126" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7027,10 +7059,10 @@
         <v>124</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>51</v>
+        <v>743</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>317</v>
+        <v>753</v>
       </c>
       <c r="D126" s="7" t="s">
         <v>149</v>
@@ -7041,33 +7073,28 @@
         <v>125</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>318</v>
+        <v>288</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="D127" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E127">
-        <v>103</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="D127" s="7"/>
     </row>
     <row r="128" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A128" s="3">
         <v>126</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D128" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E128">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="129" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7075,16 +7102,16 @@
         <v>127</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>53</v>
+        <v>316</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D129" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E129">
-        <v>59</v>
+        <v>80</v>
       </c>
     </row>
     <row r="130" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7092,16 +7119,13 @@
         <v>128</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>127</v>
+        <v>317</v>
       </c>
       <c r="D130" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="E130">
-        <v>55</v>
       </c>
     </row>
     <row r="131" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7109,16 +7133,16 @@
         <v>129</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>55</v>
+        <v>318</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>128</v>
+        <v>319</v>
       </c>
       <c r="D131" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E131">
-        <v>68</v>
+        <v>107</v>
       </c>
     </row>
     <row r="132" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7126,16 +7150,16 @@
         <v>130</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D132" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E132">
-        <v>66</v>
+        <v>57</v>
       </c>
     </row>
     <row r="133" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7143,16 +7167,16 @@
         <v>131</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D133" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E133">
-        <v>80</v>
+        <v>63</v>
       </c>
     </row>
     <row r="134" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7160,16 +7184,16 @@
         <v>132</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D134" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E134">
-        <v>37</v>
+        <v>59</v>
       </c>
     </row>
     <row r="135" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7177,16 +7201,16 @@
         <v>133</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D135" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E135">
-        <v>38</v>
+        <v>72</v>
       </c>
     </row>
     <row r="136" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7194,16 +7218,16 @@
         <v>134</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D136" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E136">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="137" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7211,16 +7235,16 @@
         <v>135</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D137" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E137">
-        <v>67</v>
+        <v>84</v>
       </c>
     </row>
     <row r="138" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7228,16 +7252,16 @@
         <v>136</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D138" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E138">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="139" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7245,16 +7269,16 @@
         <v>137</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D139" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E139">
-        <v>62</v>
+        <v>42</v>
       </c>
     </row>
     <row r="140" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7262,10 +7286,10 @@
         <v>138</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D140" s="7" t="s">
         <v>149</v>
@@ -7279,10 +7303,10 @@
         <v>139</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>320</v>
+        <v>61</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>321</v>
+        <v>134</v>
       </c>
       <c r="D141" s="7" t="s">
         <v>149</v>
@@ -7296,16 +7320,16 @@
         <v>140</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D142" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E142">
-        <v>84</v>
+        <v>53</v>
       </c>
     </row>
     <row r="143" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7313,16 +7337,16 @@
         <v>141</v>
       </c>
       <c r="B143" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D143" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E143">
         <v>66</v>
-      </c>
-      <c r="C143" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D143" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E143">
-        <v>52</v>
       </c>
     </row>
     <row r="144" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7330,16 +7354,16 @@
         <v>142</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D144" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E144">
-        <v>73</v>
+        <v>62</v>
       </c>
     </row>
     <row r="145" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7347,16 +7371,16 @@
         <v>143</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>68</v>
+        <v>320</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>141</v>
+        <v>321</v>
       </c>
       <c r="D145" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E145">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="146" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7364,16 +7388,16 @@
         <v>144</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D146" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E146">
-        <v>75</v>
+        <v>88</v>
       </c>
     </row>
     <row r="147" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -7381,49 +7405,120 @@
         <v>145</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D147" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E147">
-        <v>74</v>
+        <v>56</v>
       </c>
     </row>
     <row r="148" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A148" s="3">
         <v>146</v>
       </c>
-      <c r="B148" s="17" t="s">
+      <c r="B148" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D148" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E148">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A149" s="3">
+        <v>147</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D149" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E149">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A150" s="3">
+        <v>148</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D150" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E150">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A151" s="3">
+        <v>149</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D151" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E151">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A152" s="3">
+        <v>150</v>
+      </c>
+      <c r="B152" s="17" t="s">
         <v>322</v>
       </c>
-      <c r="C148" s="3" t="s">
+      <c r="C152" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D148" s="7"/>
-      <c r="E148">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="149" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A149" s="8">
-        <v>147</v>
-      </c>
-      <c r="B149" s="9" t="s">
+      <c r="D152" s="7"/>
+      <c r="E152">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A153" s="8">
+        <v>151</v>
+      </c>
+      <c r="B153" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="C149" s="8" t="s">
+      <c r="C153" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="D149" s="7"/>
-      <c r="E149">
+      <c r="D153" s="7"/>
+      <c r="E153">
         <v>14</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E153">
+    <sortCondition ref="A1:A153"/>
+  </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9709,6 +9804,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E160">
+    <sortCondition ref="A1:A160"/>
+  </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -10565,7 +10663,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A51E86A-E436-491E-8E79-A2D2CA117759}">
-  <dimension ref="A1:E142"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
@@ -10881,7 +10979,7 @@
         <v>149</v>
       </c>
       <c r="E20">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -10898,7 +10996,7 @@
         <v>149</v>
       </c>
       <c r="E21">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -10932,7 +11030,7 @@
         <v>149</v>
       </c>
       <c r="E23">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -10949,7 +11047,7 @@
         <v>149</v>
       </c>
       <c r="E24">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -10966,7 +11064,7 @@
         <v>149</v>
       </c>
       <c r="E25">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -10983,7 +11081,7 @@
         <v>149</v>
       </c>
       <c r="E26">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11000,7 +11098,7 @@
         <v>149</v>
       </c>
       <c r="E27">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11017,7 +11115,7 @@
         <v>149</v>
       </c>
       <c r="E28">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11034,7 +11132,7 @@
         <v>149</v>
       </c>
       <c r="E29">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11051,7 +11149,7 @@
         <v>149</v>
       </c>
       <c r="E30">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11068,7 +11166,7 @@
         <v>149</v>
       </c>
       <c r="E31">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11085,7 +11183,7 @@
         <v>149</v>
       </c>
       <c r="E32">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11102,7 +11200,7 @@
         <v>149</v>
       </c>
       <c r="E33">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11119,7 +11217,7 @@
         <v>149</v>
       </c>
       <c r="E34">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11136,7 +11234,7 @@
         <v>149</v>
       </c>
       <c r="E35">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11153,7 +11251,7 @@
         <v>149</v>
       </c>
       <c r="E36">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11170,7 +11268,7 @@
         <v>149</v>
       </c>
       <c r="E37">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11187,7 +11285,7 @@
         <v>149</v>
       </c>
       <c r="E38">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11204,7 +11302,7 @@
         <v>149</v>
       </c>
       <c r="E39">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11221,7 +11319,7 @@
         <v>149</v>
       </c>
       <c r="E40">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11343,7 +11441,7 @@
         <v>149</v>
       </c>
       <c r="E48">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11360,7 +11458,7 @@
         <v>149</v>
       </c>
       <c r="E49">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11377,7 +11475,7 @@
         <v>149</v>
       </c>
       <c r="E50">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11394,7 +11492,7 @@
         <v>149</v>
       </c>
       <c r="E51">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11411,7 +11509,7 @@
         <v>149</v>
       </c>
       <c r="E52">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11428,7 +11526,7 @@
         <v>149</v>
       </c>
       <c r="E53">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11445,7 +11543,7 @@
         <v>149</v>
       </c>
       <c r="E54">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11462,7 +11560,7 @@
         <v>149</v>
       </c>
       <c r="E55">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11479,7 +11577,7 @@
         <v>149</v>
       </c>
       <c r="E56">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11496,7 +11594,7 @@
         <v>149</v>
       </c>
       <c r="E57">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11513,7 +11611,7 @@
         <v>149</v>
       </c>
       <c r="E58">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11530,7 +11628,7 @@
         <v>149</v>
       </c>
       <c r="E59">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11561,7 +11659,7 @@
         <v>149</v>
       </c>
       <c r="E61">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11576,7 +11674,7 @@
       </c>
       <c r="D62" s="7"/>
       <c r="E62">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11591,7 +11689,7 @@
       </c>
       <c r="D63" s="7"/>
       <c r="E63">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11648,7 +11746,7 @@
       </c>
       <c r="D67" s="7"/>
       <c r="E67">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11663,7 +11761,7 @@
       </c>
       <c r="D68" s="7"/>
       <c r="E68">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11720,7 +11818,7 @@
       </c>
       <c r="D72" s="7"/>
       <c r="E72">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11735,7 +11833,7 @@
       </c>
       <c r="D73" s="7"/>
       <c r="E73">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11792,7 +11890,7 @@
       </c>
       <c r="D77" s="7"/>
       <c r="E77">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11807,7 +11905,7 @@
       </c>
       <c r="D78" s="7"/>
       <c r="E78">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11864,7 +11962,7 @@
       </c>
       <c r="D82" s="7"/>
       <c r="E82">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11879,7 +11977,7 @@
       </c>
       <c r="D83" s="7"/>
       <c r="E83">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11936,7 +12034,7 @@
       </c>
       <c r="D87" s="7"/>
       <c r="E87">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -11951,7 +12049,7 @@
       </c>
       <c r="D88" s="7"/>
       <c r="E88">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12008,7 +12106,7 @@
       </c>
       <c r="D92" s="7"/>
       <c r="E92">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12023,7 +12121,7 @@
       </c>
       <c r="D93" s="7"/>
       <c r="E93">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="94" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12040,7 +12138,7 @@
         <v>149</v>
       </c>
       <c r="E94">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12057,7 +12155,7 @@
         <v>149</v>
       </c>
       <c r="E95">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12074,7 +12172,7 @@
         <v>149</v>
       </c>
       <c r="E96">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12202,27 +12300,29 @@
         <v>103</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>734</v>
+        <v>1008</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>744</v>
-      </c>
-      <c r="D105" s="7" t="s">
-        <v>149</v>
+        <v>1012</v>
+      </c>
+      <c r="D105" s="7"/>
+      <c r="E105">
+        <v>32</v>
       </c>
     </row>
     <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A106" s="3">
         <v>104</v>
       </c>
-      <c r="B106" s="4" t="s">
-        <v>735</v>
+      <c r="B106" s="17" t="s">
+        <v>1009</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>745</v>
-      </c>
-      <c r="D106" s="7" t="s">
-        <v>149</v>
+        <v>1013</v>
+      </c>
+      <c r="D106" s="7"/>
+      <c r="E106">
+        <v>33</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12230,27 +12330,29 @@
         <v>105</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>736</v>
+        <v>1010</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>746</v>
-      </c>
-      <c r="D107" s="7" t="s">
-        <v>149</v>
+        <v>1014</v>
+      </c>
+      <c r="D107" s="7"/>
+      <c r="E107">
+        <v>34</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
         <v>106</v>
       </c>
-      <c r="B108" s="4" t="s">
-        <v>737</v>
+      <c r="B108" s="17" t="s">
+        <v>1011</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>747</v>
-      </c>
-      <c r="D108" s="7" t="s">
-        <v>149</v>
+        <v>1015</v>
+      </c>
+      <c r="D108" s="7"/>
+      <c r="E108">
+        <v>35</v>
       </c>
     </row>
     <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12258,10 +12360,10 @@
         <v>107</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="D109" s="7" t="s">
         <v>149</v>
@@ -12272,10 +12374,10 @@
         <v>108</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="D110" s="7" t="s">
         <v>149</v>
@@ -12286,10 +12388,10 @@
         <v>109</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="D111" s="7" t="s">
         <v>149</v>
@@ -12300,10 +12402,10 @@
         <v>110</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="D112" s="7" t="s">
         <v>149</v>
@@ -12314,10 +12416,10 @@
         <v>111</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="D113" s="7" t="s">
         <v>149</v>
@@ -12328,10 +12430,10 @@
         <v>112</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="D114" s="7" t="s">
         <v>149</v>
@@ -12342,14 +12444,13 @@
         <v>113</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>288</v>
+        <v>740</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D115" s="7"/>
-      <c r="E115">
-        <v>1</v>
+        <v>750</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12357,16 +12458,13 @@
         <v>114</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>50</v>
+        <v>741</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>123</v>
+        <v>751</v>
       </c>
       <c r="D116" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="E116">
-        <v>49</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12374,16 +12472,13 @@
         <v>115</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>316</v>
+        <v>742</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>124</v>
+        <v>752</v>
       </c>
       <c r="D117" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="E117">
-        <v>75</v>
       </c>
     </row>
     <row r="118" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12391,16 +12486,13 @@
         <v>116</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>51</v>
+        <v>743</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>317</v>
+        <v>753</v>
       </c>
       <c r="D118" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="E118">
-        <v>106</v>
       </c>
     </row>
     <row r="119" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12408,16 +12500,14 @@
         <v>117</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>318</v>
+        <v>288</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="D119" s="7" t="s">
-        <v>149</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="D119" s="7"/>
       <c r="E119">
-        <v>102</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12425,16 +12515,16 @@
         <v>118</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D120" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E120">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="121" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12442,16 +12532,16 @@
         <v>119</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>53</v>
+        <v>316</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D121" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E121">
-        <v>58</v>
+        <v>79</v>
       </c>
     </row>
     <row r="122" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12459,16 +12549,16 @@
         <v>120</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>127</v>
+        <v>317</v>
       </c>
       <c r="D122" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E122">
-        <v>54</v>
+        <v>110</v>
       </c>
     </row>
     <row r="123" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12476,16 +12566,16 @@
         <v>121</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>55</v>
+        <v>318</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>128</v>
+        <v>319</v>
       </c>
       <c r="D123" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E123">
-        <v>67</v>
+        <v>106</v>
       </c>
     </row>
     <row r="124" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12493,16 +12583,16 @@
         <v>122</v>
       </c>
       <c r="B124" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D124" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E124">
         <v>56</v>
-      </c>
-      <c r="C124" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D124" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E124">
-        <v>65</v>
       </c>
     </row>
     <row r="125" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12510,16 +12600,16 @@
         <v>123</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D125" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E125">
-        <v>79</v>
+        <v>62</v>
       </c>
     </row>
     <row r="126" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12527,16 +12617,16 @@
         <v>124</v>
       </c>
       <c r="B126" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D126" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E126">
         <v>58</v>
-      </c>
-      <c r="C126" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="D126" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E126">
-        <v>36</v>
       </c>
     </row>
     <row r="127" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12544,16 +12634,16 @@
         <v>125</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D127" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E127">
-        <v>37</v>
+        <v>71</v>
       </c>
     </row>
     <row r="128" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12561,16 +12651,16 @@
         <v>126</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D128" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E128">
-        <v>53</v>
+        <v>69</v>
       </c>
     </row>
     <row r="129" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12578,16 +12668,16 @@
         <v>127</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D129" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E129">
-        <v>66</v>
+        <v>83</v>
       </c>
     </row>
     <row r="130" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12595,16 +12685,16 @@
         <v>128</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D130" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E130">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="131" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12612,16 +12702,16 @@
         <v>129</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D131" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E131">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="132" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12629,10 +12719,10 @@
         <v>130</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D132" s="7" t="s">
         <v>149</v>
@@ -12646,10 +12736,10 @@
         <v>131</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>320</v>
+        <v>61</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>321</v>
+        <v>134</v>
       </c>
       <c r="D133" s="7" t="s">
         <v>149</v>
@@ -12663,16 +12753,16 @@
         <v>132</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D134" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E134">
-        <v>83</v>
+        <v>52</v>
       </c>
     </row>
     <row r="135" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12680,16 +12770,16 @@
         <v>133</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D135" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E135">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="136" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12697,16 +12787,16 @@
         <v>134</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D136" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E136">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="137" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12714,16 +12804,16 @@
         <v>135</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>68</v>
+        <v>320</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>141</v>
+        <v>321</v>
       </c>
       <c r="D137" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E137">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="138" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12731,16 +12821,16 @@
         <v>136</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D138" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E138">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="139" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -12748,64 +12838,135 @@
         <v>137</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D139" s="7" t="s">
         <v>149</v>
       </c>
       <c r="E139">
-        <v>73</v>
+        <v>55</v>
       </c>
     </row>
     <row r="140" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A140" s="3">
         <v>138</v>
       </c>
-      <c r="B140" s="17" t="s">
+      <c r="B140" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D140" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E140">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A141" s="3">
+        <v>139</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D141" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E141">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A142" s="3">
+        <v>140</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D142" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E142">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A143" s="3">
+        <v>141</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D143" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E143">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A144" s="3">
+        <v>142</v>
+      </c>
+      <c r="B144" s="17" t="s">
         <v>322</v>
       </c>
-      <c r="C140" s="3" t="s">
+      <c r="C144" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D140" s="7"/>
-      <c r="E140">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="141" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A141" s="23">
-        <v>139</v>
-      </c>
-      <c r="B141" s="24" t="s">
+      <c r="D144" s="7"/>
+      <c r="E144">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A145" s="23">
+        <v>143</v>
+      </c>
+      <c r="B145" s="24" t="s">
         <v>295</v>
       </c>
-      <c r="C141" s="23" t="s">
+      <c r="C145" s="23" t="s">
         <v>296</v>
       </c>
-      <c r="D141" s="7"/>
-      <c r="E141">
+      <c r="D145" s="7"/>
+      <c r="E145">
         <v>12</v>
       </c>
     </row>
-    <row r="142" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A142" s="23">
-        <v>140</v>
-      </c>
-      <c r="B142" s="24" t="s">
+    <row r="146" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A146" s="23">
+        <v>144</v>
+      </c>
+      <c r="B146" s="24" t="s">
         <v>297</v>
       </c>
-      <c r="C142" s="23" t="s">
+      <c r="C146" s="23" t="s">
         <v>239</v>
       </c>
-      <c r="D142" s="7"/>
-      <c r="E142">
+      <c r="D146" s="7"/>
+      <c r="E146">
         <v>13</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E146">
+    <sortCondition ref="A1:A146"/>
+  </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>